<commit_message>
Fix calls from dashboard, linting.
</commit_message>
<xml_diff>
--- a/api/templates/xdr_devices_summary/en.xlsx
+++ b/api/templates/xdr_devices_summary/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/xdr_devices_summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72E783B-146F-F841-9AA8-7A4AEC9248E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587420F8-A095-3346-9832-EBBE579CC1C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -101,12 +101,6 @@
     <t>&lt;locationName&gt;</t>
   </si>
   <si>
-    <t>&lt;totalPmdtSites&gt;</t>
-  </si>
-  <si>
-    <t>&lt;totalXdrSites&gt;</t>
-  </si>
-  <si>
     <t>&lt;cntAll&gt;</t>
   </si>
   <si>
@@ -132,6 +126,12 @@
   </si>
   <si>
     <t>&lt;cnt_NoResult&gt;</t>
+  </si>
+  <si>
+    <t>&lt;hasPerformedXdr&gt;</t>
+  </si>
+  <si>
+    <t>&lt;isPmdt&gt;</t>
   </si>
 </sst>
 </file>
@@ -265,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -274,10 +274,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -293,6 +289,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -696,29 +697,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="9" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
     </row>
-    <row r="5" spans="1:17" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:17" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -761,13 +787,13 @@
         <v>14</v>
       </c>
       <c r="N8" s="1"/>
-      <c r="O8" s="6" t="s">
+      <c r="O8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="P8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q8" s="6" t="s">
+      <c r="Q8" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -776,43 +802,43 @@
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="M9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="N9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="10" t="s">
+      <c r="O9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="P9" s="10" t="s">
+      <c r="P9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="Q9" s="10" t="s">
+      <c r="Q9" s="8" t="s">
         <v>18</v>
       </c>
     </row>
@@ -821,65 +847,70 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>22</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" t="s">
-        <v>24</v>
       </c>
       <c r="F10" s="3" t="e">
         <f>IF(D10&gt;0, E10/D10, 0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H10" s="3" t="e">
         <f>IF(D10&gt;0, G10/D10, 0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="I10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J10" s="3" t="e">
         <f>IF(D10&gt;0, I10/D10, 0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="K10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L10" s="3" t="e">
         <f>IF(D10&gt;0, K10/D10, 0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="M10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N10" s="3" t="e">
         <f>IF(D10&gt;0, M10/D10, 0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="O10" t="s">
+        <v>27</v>
+      </c>
+      <c r="P10" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q10" t="s">
         <v>29</v>
-      </c>
-      <c r="P10" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="14">
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="M8:N8"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>

</xml_diff>